<commit_message>
Update for internal gcd function
</commit_message>
<xml_diff>
--- a/sports_scoring_criteria.xlsx
+++ b/sports_scoring_criteria.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\spr-fs-app01\collab\Mal_Share\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B0698F-833C-4F39-80D8-FC58274402E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72B341B-E147-45F5-B425-C79AB143ED45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
   </bookViews>
   <sheets>
     <sheet name="Main test items" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="125">
   <si>
     <t>Drop Jump</t>
   </si>
@@ -413,6 +413,9 @@
   <si>
     <t>Knee Flexion</t>
   </si>
+  <si>
+    <t>Note: bars out of gray boxes</t>
+  </si>
 </sst>
 </file>
 
@@ -526,7 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -603,10 +606,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -44599,8 +44605,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
-            <a:alpha val="18000"/>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:ln>
@@ -44755,13 +44761,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>79945</xdr:colOff>
+      <xdr:colOff>175195</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>141415</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>286689</xdr:colOff>
+      <xdr:colOff>381939</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>67013</xdr:rowOff>
     </xdr:to>
@@ -44792,12 +44798,17 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="6316124" y="4858986"/>
-          <a:ext cx="206744" cy="680409"/>
+          <a:off x="6404545" y="5094415"/>
+          <a:ext cx="206744" cy="687598"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -44805,13 +44816,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>934170</xdr:colOff>
+      <xdr:colOff>962745</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>116456</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1167801</xdr:colOff>
+      <xdr:colOff>1196376</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>62542</xdr:rowOff>
     </xdr:to>
@@ -44828,15 +44839,15 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3414264" y="4834027"/>
-          <a:ext cx="233631" cy="700897"/>
+          <a:off x="3439245" y="5069456"/>
+          <a:ext cx="233631" cy="708086"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
-            <a:alpha val="18000"/>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:ln>
@@ -44903,8 +44914,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
-            <a:alpha val="18000"/>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:ln>
@@ -46238,7 +46249,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -46306,7 +46318,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -46694,7 +46707,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -46762,7 +46776,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -47150,7 +47165,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -47218,7 +47234,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -49205,7 +49222,7 @@
       <sheetName val="Late Rehab Comparisons"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="0"/>
       <sheetData sheetId="1">
         <row r="1">
           <cell r="E1" t="str">
@@ -49444,11 +49461,11 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -52161,7 +52178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D2AC12-7DF8-42A5-A2D6-4F386C354C01}">
-  <dimension ref="A1:AE55"/>
+  <dimension ref="A1:AE69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="24"/>
@@ -53398,100 +53415,100 @@
     </row>
     <row r="24" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18"/>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32" t="s">
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32" t="s">
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="R24" s="32" t="s">
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+      <c r="R24" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="S24" s="32"/>
-      <c r="T24" s="32"/>
-      <c r="U24" s="32"/>
-      <c r="V24" s="32"/>
-      <c r="W24" s="32" t="s">
+      <c r="S24" s="33"/>
+      <c r="T24" s="33"/>
+      <c r="U24" s="33"/>
+      <c r="V24" s="33"/>
+      <c r="W24" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="X24" s="32"/>
-      <c r="Y24" s="32" t="s">
+      <c r="X24" s="33"/>
+      <c r="Y24" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="Z24" s="32"/>
-      <c r="AA24" s="32"/>
-      <c r="AB24" s="32"/>
-      <c r="AC24" s="32"/>
+      <c r="Z24" s="33"/>
+      <c r="AA24" s="33"/>
+      <c r="AB24" s="33"/>
+      <c r="AC24" s="33"/>
     </row>
     <row r="25" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-      <c r="T25" s="32"/>
-      <c r="U25" s="32"/>
-      <c r="V25" s="32"/>
-      <c r="W25" s="32"/>
-      <c r="X25" s="32"/>
-      <c r="Y25" s="32"/>
-      <c r="Z25" s="32"/>
-      <c r="AA25" s="32"/>
-      <c r="AB25" s="32"/>
-      <c r="AC25" s="32"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="R25" s="33"/>
+      <c r="S25" s="33"/>
+      <c r="T25" s="33"/>
+      <c r="U25" s="33"/>
+      <c r="V25" s="33"/>
+      <c r="W25" s="33"/>
+      <c r="X25" s="33"/>
+      <c r="Y25" s="33"/>
+      <c r="Z25" s="33"/>
+      <c r="AA25" s="33"/>
+      <c r="AB25" s="33"/>
+      <c r="AC25" s="33"/>
     </row>
     <row r="26" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="R26" s="33" t="s">
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="32"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="32"/>
+      <c r="R26" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="S26" s="33"/>
-      <c r="T26" s="33"/>
-      <c r="U26" s="33"/>
-      <c r="V26" s="33"/>
-      <c r="W26" s="33"/>
-      <c r="X26" s="33"/>
-      <c r="Y26" s="33"/>
-      <c r="Z26" s="33"/>
-      <c r="AA26" s="33"/>
-      <c r="AB26" s="33"/>
-      <c r="AC26" s="33"/>
+      <c r="S26" s="32"/>
+      <c r="T26" s="32"/>
+      <c r="U26" s="32"/>
+      <c r="V26" s="32"/>
+      <c r="W26" s="32"/>
+      <c r="X26" s="32"/>
+      <c r="Y26" s="32"/>
+      <c r="Z26" s="32"/>
+      <c r="AA26" s="32"/>
+      <c r="AB26" s="32"/>
+      <c r="AC26" s="32"/>
     </row>
     <row r="27" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
@@ -53526,35 +53543,35 @@
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="23"/>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="33"/>
-      <c r="J33" s="33"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+      <c r="L33" s="32"/>
+      <c r="M33" s="32"/>
       <c r="Q33" s="23"/>
-      <c r="R33" s="33" t="s">
+      <c r="R33" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="S33" s="33"/>
-      <c r="T33" s="33"/>
-      <c r="U33" s="33"/>
-      <c r="V33" s="33"/>
-      <c r="W33" s="33"/>
-      <c r="X33" s="33"/>
-      <c r="Y33" s="33"/>
-      <c r="Z33" s="33"/>
-      <c r="AA33" s="33"/>
-      <c r="AB33" s="33"/>
-      <c r="AC33" s="33"/>
+      <c r="S33" s="32"/>
+      <c r="T33" s="32"/>
+      <c r="U33" s="32"/>
+      <c r="V33" s="32"/>
+      <c r="W33" s="32"/>
+      <c r="X33" s="32"/>
+      <c r="Y33" s="32"/>
+      <c r="Z33" s="32"/>
+      <c r="AA33" s="32"/>
+      <c r="AB33" s="32"/>
+      <c r="AC33" s="32"/>
     </row>
     <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
@@ -53586,20 +53603,20 @@
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="31"/>
-      <c r="R40" s="33" t="s">
+      <c r="R40" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="S40" s="33"/>
-      <c r="T40" s="33"/>
-      <c r="U40" s="33"/>
-      <c r="V40" s="33"/>
-      <c r="W40" s="33"/>
-      <c r="X40" s="33"/>
-      <c r="Y40" s="33"/>
-      <c r="Z40" s="33"/>
-      <c r="AA40" s="33"/>
-      <c r="AB40" s="33"/>
-      <c r="AC40" s="33"/>
+      <c r="S40" s="32"/>
+      <c r="T40" s="32"/>
+      <c r="U40" s="32"/>
+      <c r="V40" s="32"/>
+      <c r="W40" s="32"/>
+      <c r="X40" s="32"/>
+      <c r="Y40" s="32"/>
+      <c r="Z40" s="32"/>
+      <c r="AA40" s="32"/>
+      <c r="AB40" s="32"/>
+      <c r="AC40" s="32"/>
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A41" s="31"/>
@@ -53609,20 +53626,20 @@
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="23"/>
-      <c r="B42" s="33" t="s">
+      <c r="B42" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
-      <c r="M42" s="33"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="32"/>
+      <c r="K42" s="32"/>
+      <c r="L42" s="32"/>
+      <c r="M42" s="32"/>
       <c r="Q42" s="31"/>
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.25">
@@ -53656,20 +53673,20 @@
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
-      <c r="B49" s="33" t="s">
+      <c r="B49" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C49" s="33"/>
-      <c r="D49" s="33"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
-      <c r="J49" s="33"/>
-      <c r="K49" s="33"/>
-      <c r="L49" s="33"/>
-      <c r="M49" s="33"/>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="32"/>
+      <c r="H49" s="32"/>
+      <c r="I49" s="32"/>
+      <c r="J49" s="32"/>
+      <c r="K49" s="32"/>
+      <c r="L49" s="32"/>
+      <c r="M49" s="32"/>
       <c r="Q49" s="31"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
@@ -53695,8 +53712,136 @@
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="31"/>
     </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B57" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="C57" s="34"/>
+      <c r="D57" s="34"/>
+      <c r="E57" s="34"/>
+      <c r="F57" s="34"/>
+      <c r="G57" s="34"/>
+      <c r="H57" s="34"/>
+      <c r="I57" s="34"/>
+      <c r="J57" s="34"/>
+      <c r="K57" s="34"/>
+      <c r="L57" s="34"/>
+      <c r="M57" s="34"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B58" s="34"/>
+      <c r="C58" s="34"/>
+      <c r="D58" s="34"/>
+      <c r="E58" s="34"/>
+      <c r="F58" s="34"/>
+      <c r="G58" s="34"/>
+      <c r="H58" s="34"/>
+      <c r="I58" s="34"/>
+      <c r="J58" s="34"/>
+      <c r="K58" s="34"/>
+      <c r="L58" s="34"/>
+      <c r="M58" s="34"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B59" s="34"/>
+      <c r="C59" s="34"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="34"/>
+      <c r="F59" s="34"/>
+      <c r="G59" s="34"/>
+      <c r="H59" s="34"/>
+      <c r="I59" s="34"/>
+      <c r="J59" s="34"/>
+      <c r="K59" s="34"/>
+      <c r="L59" s="34"/>
+      <c r="M59" s="34"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B60" s="34"/>
+      <c r="C60" s="34"/>
+      <c r="D60" s="34"/>
+      <c r="E60" s="34"/>
+      <c r="F60" s="34"/>
+      <c r="G60" s="34"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="34"/>
+      <c r="J60" s="34"/>
+      <c r="K60" s="34"/>
+      <c r="L60" s="34"/>
+      <c r="M60" s="34"/>
+    </row>
+    <row r="66" spans="18:29" x14ac:dyDescent="0.25">
+      <c r="R66" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="S66" s="34"/>
+      <c r="T66" s="34"/>
+      <c r="U66" s="34"/>
+      <c r="V66" s="34"/>
+      <c r="W66" s="34"/>
+      <c r="X66" s="34"/>
+      <c r="Y66" s="34"/>
+      <c r="Z66" s="34"/>
+      <c r="AA66" s="34"/>
+      <c r="AB66" s="34"/>
+      <c r="AC66" s="34"/>
+    </row>
+    <row r="67" spans="18:29" x14ac:dyDescent="0.25">
+      <c r="R67" s="34"/>
+      <c r="S67" s="34"/>
+      <c r="T67" s="34"/>
+      <c r="U67" s="34"/>
+      <c r="V67" s="34"/>
+      <c r="W67" s="34"/>
+      <c r="X67" s="34"/>
+      <c r="Y67" s="34"/>
+      <c r="Z67" s="34"/>
+      <c r="AA67" s="34"/>
+      <c r="AB67" s="34"/>
+      <c r="AC67" s="34"/>
+    </row>
+    <row r="68" spans="18:29" x14ac:dyDescent="0.25">
+      <c r="R68" s="34"/>
+      <c r="S68" s="34"/>
+      <c r="T68" s="34"/>
+      <c r="U68" s="34"/>
+      <c r="V68" s="34"/>
+      <c r="W68" s="34"/>
+      <c r="X68" s="34"/>
+      <c r="Y68" s="34"/>
+      <c r="Z68" s="34"/>
+      <c r="AA68" s="34"/>
+      <c r="AB68" s="34"/>
+      <c r="AC68" s="34"/>
+    </row>
+    <row r="69" spans="18:29" x14ac:dyDescent="0.25">
+      <c r="R69" s="34"/>
+      <c r="S69" s="34"/>
+      <c r="T69" s="34"/>
+      <c r="U69" s="34"/>
+      <c r="V69" s="34"/>
+      <c r="W69" s="34"/>
+      <c r="X69" s="34"/>
+      <c r="Y69" s="34"/>
+      <c r="Z69" s="34"/>
+      <c r="AA69" s="34"/>
+      <c r="AB69" s="34"/>
+      <c r="AC69" s="34"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="25">
+    <mergeCell ref="R66:AC69"/>
+    <mergeCell ref="B57:M60"/>
+    <mergeCell ref="A50:A55"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="I24:M25"/>
+    <mergeCell ref="Q27:Q32"/>
+    <mergeCell ref="B26:M26"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="Q34:Q39"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="Q47:Q52"/>
+    <mergeCell ref="B49:M49"/>
     <mergeCell ref="R21:AC23"/>
     <mergeCell ref="A27:A32"/>
     <mergeCell ref="A21:M23"/>
@@ -53710,16 +53855,6 @@
     <mergeCell ref="R24:V25"/>
     <mergeCell ref="W24:X25"/>
     <mergeCell ref="E24:H25"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="I24:M25"/>
-    <mergeCell ref="Q27:Q32"/>
-    <mergeCell ref="B26:M26"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="Q34:Q39"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="Q47:Q52"/>
-    <mergeCell ref="B49:M49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
UI and dataframe updates June 18
</commit_message>
<xml_diff>
--- a/sports_scoring_criteria.xlsx
+++ b/sports_scoring_criteria.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\spr-fs-app01\collab\Mal_Share\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72B341B-E147-45F5-B425-C79AB143ED45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497440FC-8CC9-417A-8EFE-AD74651409F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="126">
   <si>
     <t>Drop Jump</t>
   </si>
@@ -414,7 +414,10 @@
     <t>Knee Flexion</t>
   </si>
   <si>
-    <t>Note: bars out of gray boxes</t>
+    <t>NOTE: Colored bars projecting into gray areas are considered outside of the identified cut-points for each measure.</t>
+  </si>
+  <si>
+    <t>Plots are designed to be anatomically aligned such that bars point in the direction you would see the segment if looking at a photo of the movement.</t>
   </si>
 </sst>
 </file>
@@ -424,7 +427,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,6 +504,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -529,7 +541,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -606,14 +618,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1002,6 +1017,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1009,7 +1025,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1562,6 +1577,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1569,7 +1585,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2112,6 +2127,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2119,7 +2135,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2559,6 +2574,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2566,7 +2582,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3005,6 +3020,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3012,7 +3028,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5499,6 +5514,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5506,7 +5522,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6273,6 +6288,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6280,7 +6296,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6622,6 +6637,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6629,7 +6645,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6971,6 +6986,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6978,7 +6994,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7373,6 +7388,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7380,7 +7396,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7665,6 +7680,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7672,7 +7688,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8019,6 +8034,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8026,7 +8042,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8374,6 +8389,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8381,7 +8397,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8664,6 +8679,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8671,7 +8687,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9008,6 +9023,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9015,7 +9031,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9360,6 +9375,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9367,7 +9383,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9651,6 +9666,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9658,7 +9674,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10003,6 +10018,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10010,7 +10026,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10347,6 +10362,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10354,7 +10370,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10638,6 +10653,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10645,7 +10661,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10989,6 +11004,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10996,7 +11012,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11336,6 +11351,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11343,7 +11359,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11683,6 +11698,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11690,7 +11706,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11964,6 +11979,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11971,7 +11987,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12312,6 +12327,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12319,7 +12335,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12660,6 +12675,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12667,7 +12683,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12941,6 +12956,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12948,7 +12964,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13230,6 +13245,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13237,7 +13253,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13519,6 +13534,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13526,7 +13542,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13800,6 +13815,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13807,7 +13823,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14089,6 +14104,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14096,7 +14112,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14469,6 +14484,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14476,7 +14492,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14758,6 +14773,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14765,7 +14781,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15039,6 +15054,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15046,7 +15062,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15418,6 +15433,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15425,7 +15441,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15768,6 +15783,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15775,7 +15791,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16321,6 +16336,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -16328,7 +16344,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16879,6 +16894,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -16886,7 +16902,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -17231,6 +17246,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -17238,7 +17254,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -44469,7 +44484,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -44537,7 +44553,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -44723,8 +44740,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
-            <a:alpha val="18000"/>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:ln>
@@ -44761,13 +44778,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>175195</xdr:colOff>
+      <xdr:colOff>70420</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>141415</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>381939</xdr:colOff>
+      <xdr:colOff>277164</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>67013</xdr:rowOff>
     </xdr:to>
@@ -44798,17 +44815,13 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="6404545" y="5094415"/>
+          <a:off x="6299770" y="5094415"/>
           <a:ext cx="206744" cy="687598"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
+        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -45082,7 +45095,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45150,7 +45164,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45218,7 +45233,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45286,7 +45302,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45460,7 +45477,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45628,7 +45646,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45696,7 +45715,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -45764,7 +45784,8 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg2">
+          <a:schemeClr val="bg1">
+            <a:lumMod val="50000"/>
             <a:alpha val="18000"/>
           </a:schemeClr>
         </a:solidFill>
@@ -46219,15 +46240,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>142878</xdr:colOff>
+      <xdr:colOff>152403</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>134786</xdr:rowOff>
+      <xdr:rowOff>106211</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>133891</xdr:colOff>
+      <xdr:colOff>180975</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>80871</xdr:rowOff>
+      <xdr:rowOff>52296</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -46242,8 +46263,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12264788" y="6361979"/>
-          <a:ext cx="1725282" cy="700897"/>
+          <a:off x="12258678" y="6392711"/>
+          <a:ext cx="1762122" cy="708085"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -49222,7 +49243,7 @@
       <sheetName val="Late Rehab Comparisons"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1">
         <row r="1">
           <cell r="E1" t="str">
@@ -49461,11 +49482,11 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -53415,100 +53436,100 @@
     </row>
     <row r="24" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18"/>
-      <c r="B24" s="33" t="s">
+      <c r="B24" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33" t="s">
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33" t="s">
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="R24" s="33" t="s">
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="32"/>
+      <c r="R24" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="S24" s="33"/>
-      <c r="T24" s="33"/>
-      <c r="U24" s="33"/>
-      <c r="V24" s="33"/>
-      <c r="W24" s="33" t="s">
+      <c r="S24" s="32"/>
+      <c r="T24" s="32"/>
+      <c r="U24" s="32"/>
+      <c r="V24" s="32"/>
+      <c r="W24" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="X24" s="33"/>
-      <c r="Y24" s="33" t="s">
+      <c r="X24" s="32"/>
+      <c r="Y24" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="Z24" s="33"/>
-      <c r="AA24" s="33"/>
-      <c r="AB24" s="33"/>
-      <c r="AC24" s="33"/>
+      <c r="Z24" s="32"/>
+      <c r="AA24" s="32"/>
+      <c r="AB24" s="32"/>
+      <c r="AC24" s="32"/>
     </row>
     <row r="25" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="R25" s="33"/>
-      <c r="S25" s="33"/>
-      <c r="T25" s="33"/>
-      <c r="U25" s="33"/>
-      <c r="V25" s="33"/>
-      <c r="W25" s="33"/>
-      <c r="X25" s="33"/>
-      <c r="Y25" s="33"/>
-      <c r="Z25" s="33"/>
-      <c r="AA25" s="33"/>
-      <c r="AB25" s="33"/>
-      <c r="AC25" s="33"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="32"/>
+      <c r="R25" s="32"/>
+      <c r="S25" s="32"/>
+      <c r="T25" s="32"/>
+      <c r="U25" s="32"/>
+      <c r="V25" s="32"/>
+      <c r="W25" s="32"/>
+      <c r="X25" s="32"/>
+      <c r="Y25" s="32"/>
+      <c r="Z25" s="32"/>
+      <c r="AA25" s="32"/>
+      <c r="AB25" s="32"/>
+      <c r="AC25" s="32"/>
     </row>
     <row r="26" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="R26" s="32" t="s">
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
+      <c r="R26" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="S26" s="32"/>
-      <c r="T26" s="32"/>
-      <c r="U26" s="32"/>
-      <c r="V26" s="32"/>
-      <c r="W26" s="32"/>
-      <c r="X26" s="32"/>
-      <c r="Y26" s="32"/>
-      <c r="Z26" s="32"/>
-      <c r="AA26" s="32"/>
-      <c r="AB26" s="32"/>
-      <c r="AC26" s="32"/>
+      <c r="S26" s="33"/>
+      <c r="T26" s="33"/>
+      <c r="U26" s="33"/>
+      <c r="V26" s="33"/>
+      <c r="W26" s="33"/>
+      <c r="X26" s="33"/>
+      <c r="Y26" s="33"/>
+      <c r="Z26" s="33"/>
+      <c r="AA26" s="33"/>
+      <c r="AB26" s="33"/>
+      <c r="AC26" s="33"/>
     </row>
     <row r="27" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
@@ -53543,35 +53564,35 @@
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="23"/>
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="32"/>
-      <c r="K33" s="32"/>
-      <c r="L33" s="32"/>
-      <c r="M33" s="32"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="33"/>
+      <c r="J33" s="33"/>
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
       <c r="Q33" s="23"/>
-      <c r="R33" s="32" t="s">
+      <c r="R33" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="S33" s="32"/>
-      <c r="T33" s="32"/>
-      <c r="U33" s="32"/>
-      <c r="V33" s="32"/>
-      <c r="W33" s="32"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="32"/>
-      <c r="Z33" s="32"/>
-      <c r="AA33" s="32"/>
-      <c r="AB33" s="32"/>
-      <c r="AC33" s="32"/>
+      <c r="S33" s="33"/>
+      <c r="T33" s="33"/>
+      <c r="U33" s="33"/>
+      <c r="V33" s="33"/>
+      <c r="W33" s="33"/>
+      <c r="X33" s="33"/>
+      <c r="Y33" s="33"/>
+      <c r="Z33" s="33"/>
+      <c r="AA33" s="33"/>
+      <c r="AB33" s="33"/>
+      <c r="AC33" s="33"/>
     </row>
     <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
@@ -53603,20 +53624,20 @@
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="31"/>
-      <c r="R40" s="32" t="s">
+      <c r="R40" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="S40" s="32"/>
-      <c r="T40" s="32"/>
-      <c r="U40" s="32"/>
-      <c r="V40" s="32"/>
-      <c r="W40" s="32"/>
-      <c r="X40" s="32"/>
-      <c r="Y40" s="32"/>
-      <c r="Z40" s="32"/>
-      <c r="AA40" s="32"/>
-      <c r="AB40" s="32"/>
-      <c r="AC40" s="32"/>
+      <c r="S40" s="33"/>
+      <c r="T40" s="33"/>
+      <c r="U40" s="33"/>
+      <c r="V40" s="33"/>
+      <c r="W40" s="33"/>
+      <c r="X40" s="33"/>
+      <c r="Y40" s="33"/>
+      <c r="Z40" s="33"/>
+      <c r="AA40" s="33"/>
+      <c r="AB40" s="33"/>
+      <c r="AC40" s="33"/>
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A41" s="31"/>
@@ -53626,20 +53647,20 @@
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="23"/>
-      <c r="B42" s="32" t="s">
+      <c r="B42" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="32"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
       <c r="Q42" s="31"/>
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.25">
@@ -53673,20 +53694,20 @@
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
-      <c r="B49" s="32" t="s">
+      <c r="B49" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C49" s="32"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="32"/>
-      <c r="J49" s="32"/>
-      <c r="K49" s="32"/>
-      <c r="L49" s="32"/>
-      <c r="M49" s="32"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="33"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="33"/>
+      <c r="L49" s="33"/>
+      <c r="M49" s="33"/>
       <c r="Q49" s="31"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
@@ -53712,38 +53733,40 @@
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="31"/>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B57" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="C57" s="34"/>
-      <c r="D57" s="34"/>
-      <c r="E57" s="34"/>
-      <c r="F57" s="34"/>
-      <c r="G57" s="34"/>
-      <c r="H57" s="34"/>
-      <c r="I57" s="34"/>
-      <c r="J57" s="34"/>
-      <c r="K57" s="34"/>
-      <c r="L57" s="34"/>
-      <c r="M57" s="34"/>
+    <row r="57" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="C57" s="35"/>
+      <c r="D57" s="35"/>
+      <c r="E57" s="35"/>
+      <c r="F57" s="35"/>
+      <c r="G57" s="35"/>
+      <c r="H57" s="35"/>
+      <c r="I57" s="35"/>
+      <c r="J57" s="35"/>
+      <c r="K57" s="35"/>
+      <c r="L57" s="35"/>
+      <c r="M57" s="35"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B58" s="34"/>
-      <c r="C58" s="34"/>
-      <c r="D58" s="34"/>
-      <c r="E58" s="34"/>
-      <c r="F58" s="34"/>
-      <c r="G58" s="34"/>
-      <c r="H58" s="34"/>
-      <c r="I58" s="34"/>
-      <c r="J58" s="34"/>
-      <c r="K58" s="34"/>
-      <c r="L58" s="34"/>
-      <c r="M58" s="34"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="35"/>
+      <c r="D58" s="35"/>
+      <c r="E58" s="35"/>
+      <c r="F58" s="35"/>
+      <c r="G58" s="35"/>
+      <c r="H58" s="35"/>
+      <c r="I58" s="35"/>
+      <c r="J58" s="35"/>
+      <c r="K58" s="35"/>
+      <c r="L58" s="35"/>
+      <c r="M58" s="35"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B59" s="34"/>
+      <c r="B59" s="34" t="s">
+        <v>124</v>
+      </c>
       <c r="C59" s="34"/>
       <c r="D59" s="34"/>
       <c r="E59" s="34"/>
@@ -53771,37 +53794,39 @@
       <c r="M60" s="34"/>
     </row>
     <row r="66" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R66" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="S66" s="34"/>
-      <c r="T66" s="34"/>
-      <c r="U66" s="34"/>
-      <c r="V66" s="34"/>
-      <c r="W66" s="34"/>
-      <c r="X66" s="34"/>
-      <c r="Y66" s="34"/>
-      <c r="Z66" s="34"/>
-      <c r="AA66" s="34"/>
-      <c r="AB66" s="34"/>
-      <c r="AC66" s="34"/>
+      <c r="R66" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="S66" s="35"/>
+      <c r="T66" s="35"/>
+      <c r="U66" s="35"/>
+      <c r="V66" s="35"/>
+      <c r="W66" s="35"/>
+      <c r="X66" s="35"/>
+      <c r="Y66" s="35"/>
+      <c r="Z66" s="35"/>
+      <c r="AA66" s="35"/>
+      <c r="AB66" s="35"/>
+      <c r="AC66" s="35"/>
     </row>
     <row r="67" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R67" s="34"/>
-      <c r="S67" s="34"/>
-      <c r="T67" s="34"/>
-      <c r="U67" s="34"/>
-      <c r="V67" s="34"/>
-      <c r="W67" s="34"/>
-      <c r="X67" s="34"/>
-      <c r="Y67" s="34"/>
-      <c r="Z67" s="34"/>
-      <c r="AA67" s="34"/>
-      <c r="AB67" s="34"/>
-      <c r="AC67" s="34"/>
+      <c r="R67" s="35"/>
+      <c r="S67" s="35"/>
+      <c r="T67" s="35"/>
+      <c r="U67" s="35"/>
+      <c r="V67" s="35"/>
+      <c r="W67" s="35"/>
+      <c r="X67" s="35"/>
+      <c r="Y67" s="35"/>
+      <c r="Z67" s="35"/>
+      <c r="AA67" s="35"/>
+      <c r="AB67" s="35"/>
+      <c r="AC67" s="35"/>
     </row>
     <row r="68" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R68" s="34"/>
+      <c r="R68" s="34" t="s">
+        <v>124</v>
+      </c>
       <c r="S68" s="34"/>
       <c r="T68" s="34"/>
       <c r="U68" s="34"/>
@@ -53829,19 +53854,9 @@
       <c r="AC69" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="R66:AC69"/>
-    <mergeCell ref="B57:M60"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="I24:M25"/>
-    <mergeCell ref="Q27:Q32"/>
-    <mergeCell ref="B26:M26"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="Q34:Q39"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="Q47:Q52"/>
-    <mergeCell ref="B49:M49"/>
+  <mergeCells count="27">
+    <mergeCell ref="R66:AC67"/>
+    <mergeCell ref="R68:AC69"/>
     <mergeCell ref="R21:AC23"/>
     <mergeCell ref="A27:A32"/>
     <mergeCell ref="A21:M23"/>
@@ -53855,8 +53870,21 @@
     <mergeCell ref="R24:V25"/>
     <mergeCell ref="W24:X25"/>
     <mergeCell ref="E24:H25"/>
+    <mergeCell ref="A50:A55"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="I24:M25"/>
+    <mergeCell ref="Q27:Q32"/>
+    <mergeCell ref="B26:M26"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="Q34:Q39"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="Q47:Q52"/>
+    <mergeCell ref="B49:M49"/>
+    <mergeCell ref="B59:M60"/>
+    <mergeCell ref="B57:M58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changes to Summary page
</commit_message>
<xml_diff>
--- a/sports_scoring_criteria.xlsx
+++ b/sports_scoring_criteria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://shrinershospitals-my.sharepoint.com/personal/swarshauer_shrinenet_org/Documents/Documents/GitHub/Sports_Screening_ReportGenerator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497440FC-8CC9-417A-8EFE-AD74651409F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{497440FC-8CC9-417A-8EFE-AD74651409F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{618609FF-24E8-5729-96DD-7D4E4AB33958}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
+    <workbookView minimized="1" xWindow="165" yWindow="135" windowWidth="19170" windowHeight="14610" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
   </bookViews>
   <sheets>
     <sheet name="Main test items" sheetId="1" r:id="rId1"/>
@@ -609,8 +609,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -618,17 +621,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -51052,28 +51052,28 @@
         <f t="shared" si="2"/>
         <v>-2.0266666666666668</v>
       </c>
-      <c r="P9" s="29" t="s">
+      <c r="P9" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="Q9" s="29"/>
-      <c r="R9" s="29"/>
-      <c r="S9" s="29"/>
-      <c r="T9" s="29"/>
-      <c r="U9" s="29"/>
-      <c r="V9" s="29"/>
-      <c r="W9" s="29"/>
-      <c r="X9" s="29"/>
-      <c r="Z9" s="29" t="s">
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
+      <c r="S9" s="35"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="35"/>
+      <c r="V9" s="35"/>
+      <c r="W9" s="35"/>
+      <c r="X9" s="35"/>
+      <c r="Z9" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="AA9" s="29"/>
-      <c r="AB9" s="29"/>
-      <c r="AC9" s="29"/>
-      <c r="AD9" s="29"/>
-      <c r="AE9" s="29"/>
-      <c r="AF9" s="29"/>
-      <c r="AG9" s="29"/>
-      <c r="AH9" s="29"/>
+      <c r="AA9" s="35"/>
+      <c r="AB9" s="35"/>
+      <c r="AC9" s="35"/>
+      <c r="AD9" s="35"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="35"/>
+      <c r="AG9" s="35"/>
+      <c r="AH9" s="35"/>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
@@ -51114,24 +51114,24 @@
         <f t="shared" si="2"/>
         <v>-0.45666666666666672</v>
       </c>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="29"/>
-      <c r="R10" s="29"/>
-      <c r="S10" s="29"/>
-      <c r="T10" s="29"/>
-      <c r="U10" s="29"/>
-      <c r="V10" s="29"/>
-      <c r="W10" s="29"/>
-      <c r="X10" s="29"/>
-      <c r="Z10" s="29"/>
-      <c r="AA10" s="29"/>
-      <c r="AB10" s="29"/>
-      <c r="AC10" s="29"/>
-      <c r="AD10" s="29"/>
-      <c r="AE10" s="29"/>
-      <c r="AF10" s="29"/>
-      <c r="AG10" s="29"/>
-      <c r="AH10" s="29"/>
+      <c r="P10" s="35"/>
+      <c r="Q10" s="35"/>
+      <c r="R10" s="35"/>
+      <c r="S10" s="35"/>
+      <c r="T10" s="35"/>
+      <c r="U10" s="35"/>
+      <c r="V10" s="35"/>
+      <c r="W10" s="35"/>
+      <c r="X10" s="35"/>
+      <c r="Z10" s="35"/>
+      <c r="AA10" s="35"/>
+      <c r="AB10" s="35"/>
+      <c r="AC10" s="35"/>
+      <c r="AD10" s="35"/>
+      <c r="AE10" s="35"/>
+      <c r="AF10" s="35"/>
+      <c r="AG10" s="35"/>
+      <c r="AH10" s="35"/>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="D11" s="15" t="s">
@@ -51358,89 +51358,89 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="30"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="30"/>
-      <c r="K22" s="30"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="30"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
     </row>
     <row r="34" spans="16:35" x14ac:dyDescent="0.25">
-      <c r="P34" s="29" t="s">
+      <c r="P34" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="Q34" s="29"/>
-      <c r="R34" s="29"/>
-      <c r="S34" s="29"/>
-      <c r="T34" s="29"/>
-      <c r="U34" s="29"/>
-      <c r="V34" s="29"/>
-      <c r="W34" s="29"/>
-      <c r="X34" s="29"/>
-      <c r="AA34" s="29" t="s">
+      <c r="Q34" s="35"/>
+      <c r="R34" s="35"/>
+      <c r="S34" s="35"/>
+      <c r="T34" s="35"/>
+      <c r="U34" s="35"/>
+      <c r="V34" s="35"/>
+      <c r="W34" s="35"/>
+      <c r="X34" s="35"/>
+      <c r="AA34" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="AB34" s="29"/>
-      <c r="AC34" s="29"/>
-      <c r="AD34" s="29"/>
-      <c r="AE34" s="29"/>
-      <c r="AF34" s="29"/>
-      <c r="AG34" s="29"/>
-      <c r="AH34" s="29"/>
-      <c r="AI34" s="29"/>
+      <c r="AB34" s="35"/>
+      <c r="AC34" s="35"/>
+      <c r="AD34" s="35"/>
+      <c r="AE34" s="35"/>
+      <c r="AF34" s="35"/>
+      <c r="AG34" s="35"/>
+      <c r="AH34" s="35"/>
+      <c r="AI34" s="35"/>
     </row>
     <row r="35" spans="16:35" x14ac:dyDescent="0.25">
-      <c r="P35" s="29"/>
-      <c r="Q35" s="29"/>
-      <c r="R35" s="29"/>
-      <c r="S35" s="29"/>
-      <c r="T35" s="29"/>
-      <c r="U35" s="29"/>
-      <c r="V35" s="29"/>
-      <c r="W35" s="29"/>
-      <c r="X35" s="29"/>
-      <c r="AA35" s="29"/>
-      <c r="AB35" s="29"/>
-      <c r="AC35" s="29"/>
-      <c r="AD35" s="29"/>
-      <c r="AE35" s="29"/>
-      <c r="AF35" s="29"/>
-      <c r="AG35" s="29"/>
-      <c r="AH35" s="29"/>
-      <c r="AI35" s="29"/>
+      <c r="P35" s="35"/>
+      <c r="Q35" s="35"/>
+      <c r="R35" s="35"/>
+      <c r="S35" s="35"/>
+      <c r="T35" s="35"/>
+      <c r="U35" s="35"/>
+      <c r="V35" s="35"/>
+      <c r="W35" s="35"/>
+      <c r="X35" s="35"/>
+      <c r="AA35" s="35"/>
+      <c r="AB35" s="35"/>
+      <c r="AC35" s="35"/>
+      <c r="AD35" s="35"/>
+      <c r="AE35" s="35"/>
+      <c r="AF35" s="35"/>
+      <c r="AG35" s="35"/>
+      <c r="AH35" s="35"/>
+      <c r="AI35" s="35"/>
     </row>
     <row r="36" spans="16:35" x14ac:dyDescent="0.25">
       <c r="Q36" t="s">
@@ -51844,28 +51844,28 @@
       </c>
     </row>
     <row r="59" spans="27:35" x14ac:dyDescent="0.25">
-      <c r="AA59" s="29" t="s">
+      <c r="AA59" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="AB59" s="29"/>
-      <c r="AC59" s="29"/>
-      <c r="AD59" s="29"/>
-      <c r="AE59" s="29"/>
-      <c r="AF59" s="29"/>
-      <c r="AG59" s="29"/>
-      <c r="AH59" s="29"/>
-      <c r="AI59" s="29"/>
+      <c r="AB59" s="35"/>
+      <c r="AC59" s="35"/>
+      <c r="AD59" s="35"/>
+      <c r="AE59" s="35"/>
+      <c r="AF59" s="35"/>
+      <c r="AG59" s="35"/>
+      <c r="AH59" s="35"/>
+      <c r="AI59" s="35"/>
     </row>
     <row r="60" spans="27:35" x14ac:dyDescent="0.25">
-      <c r="AA60" s="29"/>
-      <c r="AB60" s="29"/>
-      <c r="AC60" s="29"/>
-      <c r="AD60" s="29"/>
-      <c r="AE60" s="29"/>
-      <c r="AF60" s="29"/>
-      <c r="AG60" s="29"/>
-      <c r="AH60" s="29"/>
-      <c r="AI60" s="29"/>
+      <c r="AA60" s="35"/>
+      <c r="AB60" s="35"/>
+      <c r="AC60" s="35"/>
+      <c r="AD60" s="35"/>
+      <c r="AE60" s="35"/>
+      <c r="AF60" s="35"/>
+      <c r="AG60" s="35"/>
+      <c r="AH60" s="35"/>
+      <c r="AI60" s="35"/>
     </row>
     <row r="61" spans="27:35" x14ac:dyDescent="0.25">
       <c r="AB61" t="s">
@@ -53350,155 +53350,155 @@
       </c>
     </row>
     <row r="21" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="30"/>
-      <c r="L21" s="30"/>
-      <c r="M21" s="30"/>
-      <c r="R21" s="30" t="s">
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="R21" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="S21" s="30"/>
-      <c r="T21" s="30"/>
-      <c r="U21" s="30"/>
-      <c r="V21" s="30"/>
-      <c r="W21" s="30"/>
-      <c r="X21" s="30"/>
-      <c r="Y21" s="30"/>
-      <c r="Z21" s="30"/>
-      <c r="AA21" s="30"/>
-      <c r="AB21" s="30"/>
-      <c r="AC21" s="30"/>
+      <c r="S21" s="31"/>
+      <c r="T21" s="31"/>
+      <c r="U21" s="31"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="31"/>
+      <c r="X21" s="31"/>
+      <c r="Y21" s="31"/>
+      <c r="Z21" s="31"/>
+      <c r="AA21" s="31"/>
+      <c r="AB21" s="31"/>
+      <c r="AC21" s="31"/>
     </row>
     <row r="22" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="30"/>
-      <c r="K22" s="30"/>
-      <c r="L22" s="30"/>
-      <c r="M22" s="30"/>
-      <c r="R22" s="30"/>
-      <c r="S22" s="30"/>
-      <c r="T22" s="30"/>
-      <c r="U22" s="30"/>
-      <c r="V22" s="30"/>
-      <c r="W22" s="30"/>
-      <c r="X22" s="30"/>
-      <c r="Y22" s="30"/>
-      <c r="Z22" s="30"/>
-      <c r="AA22" s="30"/>
-      <c r="AB22" s="30"/>
-      <c r="AC22" s="30"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
+      <c r="M22" s="31"/>
+      <c r="R22" s="31"/>
+      <c r="S22" s="31"/>
+      <c r="T22" s="31"/>
+      <c r="U22" s="31"/>
+      <c r="V22" s="31"/>
+      <c r="W22" s="31"/>
+      <c r="X22" s="31"/>
+      <c r="Y22" s="31"/>
+      <c r="Z22" s="31"/>
+      <c r="AA22" s="31"/>
+      <c r="AB22" s="31"/>
+      <c r="AC22" s="31"/>
     </row>
     <row r="23" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="30"/>
-      <c r="K23" s="30"/>
-      <c r="L23" s="30"/>
-      <c r="M23" s="30"/>
-      <c r="R23" s="30"/>
-      <c r="S23" s="30"/>
-      <c r="T23" s="30"/>
-      <c r="U23" s="30"/>
-      <c r="V23" s="30"/>
-      <c r="W23" s="30"/>
-      <c r="X23" s="30"/>
-      <c r="Y23" s="30"/>
-      <c r="Z23" s="30"/>
-      <c r="AA23" s="30"/>
-      <c r="AB23" s="30"/>
-      <c r="AC23" s="30"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="31"/>
+      <c r="M23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31"/>
+      <c r="T23" s="31"/>
+      <c r="U23" s="31"/>
+      <c r="V23" s="31"/>
+      <c r="W23" s="31"/>
+      <c r="X23" s="31"/>
+      <c r="Y23" s="31"/>
+      <c r="Z23" s="31"/>
+      <c r="AA23" s="31"/>
+      <c r="AB23" s="31"/>
+      <c r="AC23" s="31"/>
     </row>
     <row r="24" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18"/>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32" t="s">
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32" t="s">
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="R24" s="32" t="s">
+      <c r="J24" s="34"/>
+      <c r="K24" s="34"/>
+      <c r="L24" s="34"/>
+      <c r="M24" s="34"/>
+      <c r="R24" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="S24" s="32"/>
-      <c r="T24" s="32"/>
-      <c r="U24" s="32"/>
-      <c r="V24" s="32"/>
-      <c r="W24" s="32" t="s">
+      <c r="S24" s="34"/>
+      <c r="T24" s="34"/>
+      <c r="U24" s="34"/>
+      <c r="V24" s="34"/>
+      <c r="W24" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="X24" s="32"/>
-      <c r="Y24" s="32" t="s">
+      <c r="X24" s="34"/>
+      <c r="Y24" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="Z24" s="32"/>
-      <c r="AA24" s="32"/>
-      <c r="AB24" s="32"/>
-      <c r="AC24" s="32"/>
+      <c r="Z24" s="34"/>
+      <c r="AA24" s="34"/>
+      <c r="AB24" s="34"/>
+      <c r="AC24" s="34"/>
     </row>
     <row r="25" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-      <c r="T25" s="32"/>
-      <c r="U25" s="32"/>
-      <c r="V25" s="32"/>
-      <c r="W25" s="32"/>
-      <c r="X25" s="32"/>
-      <c r="Y25" s="32"/>
-      <c r="Z25" s="32"/>
-      <c r="AA25" s="32"/>
-      <c r="AB25" s="32"/>
-      <c r="AC25" s="32"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34"/>
+      <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
+      <c r="M25" s="34"/>
+      <c r="R25" s="34"/>
+      <c r="S25" s="34"/>
+      <c r="T25" s="34"/>
+      <c r="U25" s="34"/>
+      <c r="V25" s="34"/>
+      <c r="W25" s="34"/>
+      <c r="X25" s="34"/>
+      <c r="Y25" s="34"/>
+      <c r="Z25" s="34"/>
+      <c r="AA25" s="34"/>
+      <c r="AB25" s="34"/>
+      <c r="AC25" s="34"/>
     </row>
     <row r="26" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
@@ -53532,35 +53532,35 @@
       <c r="AC26" s="33"/>
     </row>
     <row r="27" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="32" t="s">
         <v>72</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
       <c r="D27" s="20"/>
-      <c r="Q27" s="31" t="s">
+      <c r="Q27" s="32" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A28" s="31"/>
-      <c r="Q28" s="31"/>
+      <c r="A28" s="32"/>
+      <c r="Q28" s="32"/>
     </row>
     <row r="29" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A29" s="31"/>
-      <c r="Q29" s="31"/>
+      <c r="A29" s="32"/>
+      <c r="Q29" s="32"/>
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A30" s="31"/>
-      <c r="Q30" s="31"/>
+      <c r="A30" s="32"/>
+      <c r="Q30" s="32"/>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A31" s="31"/>
-      <c r="Q31" s="31"/>
+      <c r="A31" s="32"/>
+      <c r="Q31" s="32"/>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A32" s="31"/>
-      <c r="Q32" s="31"/>
+      <c r="A32" s="32"/>
+      <c r="Q32" s="32"/>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="23"/>
@@ -53595,35 +53595,35 @@
       <c r="AC33" s="33"/>
     </row>
     <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
+      <c r="A34" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="Q34" s="31" t="s">
+      <c r="Q34" s="32" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A35" s="31"/>
-      <c r="Q35" s="31"/>
+      <c r="A35" s="32"/>
+      <c r="Q35" s="32"/>
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="Q36" s="31"/>
+      <c r="A36" s="32"/>
+      <c r="Q36" s="32"/>
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A37" s="31"/>
-      <c r="Q37" s="31"/>
+      <c r="A37" s="32"/>
+      <c r="Q37" s="32"/>
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A38" s="31"/>
-      <c r="Q38" s="31"/>
+      <c r="A38" s="32"/>
+      <c r="Q38" s="32"/>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-      <c r="Q39" s="31"/>
+      <c r="A39" s="32"/>
+      <c r="Q39" s="32"/>
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A40" s="31"/>
+      <c r="A40" s="32"/>
       <c r="R40" s="33" t="s">
         <v>0</v>
       </c>
@@ -53640,8 +53640,8 @@
       <c r="AC40" s="33"/>
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A41" s="31"/>
-      <c r="Q41" s="31" t="s">
+      <c r="A41" s="32"/>
+      <c r="Q41" s="32" t="s">
         <v>122</v>
       </c>
     </row>
@@ -53661,36 +53661,36 @@
       <c r="K42" s="33"/>
       <c r="L42" s="33"/>
       <c r="M42" s="33"/>
-      <c r="Q42" s="31"/>
+      <c r="Q42" s="32"/>
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A43" s="31" t="s">
+      <c r="A43" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="Q43" s="31"/>
+      <c r="Q43" s="32"/>
     </row>
     <row r="44" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A44" s="31"/>
-      <c r="Q44" s="31"/>
+      <c r="A44" s="32"/>
+      <c r="Q44" s="32"/>
     </row>
     <row r="45" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A45" s="31"/>
+      <c r="A45" s="32"/>
       <c r="P45" s="27"/>
-      <c r="Q45" s="31"/>
+      <c r="Q45" s="32"/>
     </row>
     <row r="46" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A46" s="31"/>
-      <c r="Q46" s="31"/>
+      <c r="A46" s="32"/>
+      <c r="Q46" s="32"/>
     </row>
     <row r="47" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A47" s="31"/>
-      <c r="Q47" s="31" t="s">
+      <c r="A47" s="32"/>
+      <c r="Q47" s="32" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A48" s="31"/>
-      <c r="Q48" s="31"/>
+      <c r="A48" s="32"/>
+      <c r="Q48" s="32"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
@@ -53708,153 +53708,164 @@
       <c r="K49" s="33"/>
       <c r="L49" s="33"/>
       <c r="M49" s="33"/>
-      <c r="Q49" s="31"/>
+      <c r="Q49" s="32"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="31" t="s">
+      <c r="A50" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="Q50" s="31"/>
+      <c r="Q50" s="32"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="31"/>
-      <c r="Q51" s="31"/>
+      <c r="A51" s="32"/>
+      <c r="Q51" s="32"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="31"/>
-      <c r="Q52" s="31"/>
+      <c r="A52" s="32"/>
+      <c r="Q52" s="32"/>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="31"/>
+      <c r="A53" s="32"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="31"/>
+      <c r="A54" s="32"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A55" s="31"/>
+      <c r="A55" s="32"/>
     </row>
     <row r="57" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="35" t="s">
+      <c r="B57" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="35"/>
-      <c r="H57" s="35"/>
-      <c r="I57" s="35"/>
-      <c r="J57" s="35"/>
-      <c r="K57" s="35"/>
-      <c r="L57" s="35"/>
-      <c r="M57" s="35"/>
+      <c r="C57" s="29"/>
+      <c r="D57" s="29"/>
+      <c r="E57" s="29"/>
+      <c r="F57" s="29"/>
+      <c r="G57" s="29"/>
+      <c r="H57" s="29"/>
+      <c r="I57" s="29"/>
+      <c r="J57" s="29"/>
+      <c r="K57" s="29"/>
+      <c r="L57" s="29"/>
+      <c r="M57" s="29"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B58" s="35"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
-      <c r="G58" s="35"/>
-      <c r="H58" s="35"/>
-      <c r="I58" s="35"/>
-      <c r="J58" s="35"/>
-      <c r="K58" s="35"/>
-      <c r="L58" s="35"/>
-      <c r="M58" s="35"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+      <c r="G58" s="29"/>
+      <c r="H58" s="29"/>
+      <c r="I58" s="29"/>
+      <c r="J58" s="29"/>
+      <c r="K58" s="29"/>
+      <c r="L58" s="29"/>
+      <c r="M58" s="29"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B59" s="34" t="s">
+      <c r="B59" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="34"/>
-      <c r="D59" s="34"/>
-      <c r="E59" s="34"/>
-      <c r="F59" s="34"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="34"/>
-      <c r="I59" s="34"/>
-      <c r="J59" s="34"/>
-      <c r="K59" s="34"/>
-      <c r="L59" s="34"/>
-      <c r="M59" s="34"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="30"/>
+      <c r="E59" s="30"/>
+      <c r="F59" s="30"/>
+      <c r="G59" s="30"/>
+      <c r="H59" s="30"/>
+      <c r="I59" s="30"/>
+      <c r="J59" s="30"/>
+      <c r="K59" s="30"/>
+      <c r="L59" s="30"/>
+      <c r="M59" s="30"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B60" s="34"/>
-      <c r="C60" s="34"/>
-      <c r="D60" s="34"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
-      <c r="J60" s="34"/>
-      <c r="K60" s="34"/>
-      <c r="L60" s="34"/>
-      <c r="M60" s="34"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="30"/>
+      <c r="E60" s="30"/>
+      <c r="F60" s="30"/>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="30"/>
+      <c r="J60" s="30"/>
+      <c r="K60" s="30"/>
+      <c r="L60" s="30"/>
+      <c r="M60" s="30"/>
     </row>
     <row r="66" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R66" s="35" t="s">
+      <c r="R66" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="S66" s="35"/>
-      <c r="T66" s="35"/>
-      <c r="U66" s="35"/>
-      <c r="V66" s="35"/>
-      <c r="W66" s="35"/>
-      <c r="X66" s="35"/>
-      <c r="Y66" s="35"/>
-      <c r="Z66" s="35"/>
-      <c r="AA66" s="35"/>
-      <c r="AB66" s="35"/>
-      <c r="AC66" s="35"/>
+      <c r="S66" s="29"/>
+      <c r="T66" s="29"/>
+      <c r="U66" s="29"/>
+      <c r="V66" s="29"/>
+      <c r="W66" s="29"/>
+      <c r="X66" s="29"/>
+      <c r="Y66" s="29"/>
+      <c r="Z66" s="29"/>
+      <c r="AA66" s="29"/>
+      <c r="AB66" s="29"/>
+      <c r="AC66" s="29"/>
     </row>
     <row r="67" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R67" s="35"/>
-      <c r="S67" s="35"/>
-      <c r="T67" s="35"/>
-      <c r="U67" s="35"/>
-      <c r="V67" s="35"/>
-      <c r="W67" s="35"/>
-      <c r="X67" s="35"/>
-      <c r="Y67" s="35"/>
-      <c r="Z67" s="35"/>
-      <c r="AA67" s="35"/>
-      <c r="AB67" s="35"/>
-      <c r="AC67" s="35"/>
+      <c r="R67" s="29"/>
+      <c r="S67" s="29"/>
+      <c r="T67" s="29"/>
+      <c r="U67" s="29"/>
+      <c r="V67" s="29"/>
+      <c r="W67" s="29"/>
+      <c r="X67" s="29"/>
+      <c r="Y67" s="29"/>
+      <c r="Z67" s="29"/>
+      <c r="AA67" s="29"/>
+      <c r="AB67" s="29"/>
+      <c r="AC67" s="29"/>
     </row>
     <row r="68" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R68" s="34" t="s">
+      <c r="R68" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="S68" s="34"/>
-      <c r="T68" s="34"/>
-      <c r="U68" s="34"/>
-      <c r="V68" s="34"/>
-      <c r="W68" s="34"/>
-      <c r="X68" s="34"/>
-      <c r="Y68" s="34"/>
-      <c r="Z68" s="34"/>
-      <c r="AA68" s="34"/>
-      <c r="AB68" s="34"/>
-      <c r="AC68" s="34"/>
+      <c r="S68" s="30"/>
+      <c r="T68" s="30"/>
+      <c r="U68" s="30"/>
+      <c r="V68" s="30"/>
+      <c r="W68" s="30"/>
+      <c r="X68" s="30"/>
+      <c r="Y68" s="30"/>
+      <c r="Z68" s="30"/>
+      <c r="AA68" s="30"/>
+      <c r="AB68" s="30"/>
+      <c r="AC68" s="30"/>
     </row>
     <row r="69" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R69" s="34"/>
-      <c r="S69" s="34"/>
-      <c r="T69" s="34"/>
-      <c r="U69" s="34"/>
-      <c r="V69" s="34"/>
-      <c r="W69" s="34"/>
-      <c r="X69" s="34"/>
-      <c r="Y69" s="34"/>
-      <c r="Z69" s="34"/>
-      <c r="AA69" s="34"/>
-      <c r="AB69" s="34"/>
-      <c r="AC69" s="34"/>
+      <c r="R69" s="30"/>
+      <c r="S69" s="30"/>
+      <c r="T69" s="30"/>
+      <c r="U69" s="30"/>
+      <c r="V69" s="30"/>
+      <c r="W69" s="30"/>
+      <c r="X69" s="30"/>
+      <c r="Y69" s="30"/>
+      <c r="Z69" s="30"/>
+      <c r="AA69" s="30"/>
+      <c r="AB69" s="30"/>
+      <c r="AC69" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="Q34:Q39"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="Q47:Q52"/>
+    <mergeCell ref="B49:M49"/>
+    <mergeCell ref="B59:M60"/>
+    <mergeCell ref="B57:M58"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="I24:M25"/>
+    <mergeCell ref="Q27:Q32"/>
+    <mergeCell ref="B26:M26"/>
+    <mergeCell ref="B33:M33"/>
     <mergeCell ref="R66:AC67"/>
     <mergeCell ref="R68:AC69"/>
     <mergeCell ref="R21:AC23"/>
@@ -53871,17 +53882,6 @@
     <mergeCell ref="W24:X25"/>
     <mergeCell ref="E24:H25"/>
     <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="I24:M25"/>
-    <mergeCell ref="Q27:Q32"/>
-    <mergeCell ref="B26:M26"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="Q34:Q39"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="Q47:Q52"/>
-    <mergeCell ref="B49:M49"/>
-    <mergeCell ref="B59:M60"/>
-    <mergeCell ref="B57:M58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updates to existing data check
</commit_message>
<xml_diff>
--- a/sports_scoring_criteria.xlsx
+++ b/sports_scoring_criteria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\spr-fs-app01\collab\Mal_Share\ViconDatabase\Python Code\Sports_Screening_ReportGenerator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497440FC-8CC9-417A-8EFE-AD74651409F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D229E0-478B-4680-BD6F-75F9F24F7C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{948AD37F-D091-4D2C-AFEA-0D7F44D6D79C}"/>
   </bookViews>
   <sheets>
     <sheet name="Main test items" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="126">
   <si>
     <t>Drop Jump</t>
   </si>
@@ -514,7 +514,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -524,6 +524,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -541,7 +565,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -615,20 +639,35 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1017,7 +1056,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1025,6 +1063,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1577,7 +1616,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1585,6 +1623,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2127,7 +2166,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2135,6 +2173,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2574,7 +2613,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2582,6 +2620,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3020,7 +3059,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3028,6 +3066,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5514,7 +5553,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5522,6 +5560,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6288,7 +6327,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6296,6 +6334,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6637,7 +6676,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6645,6 +6683,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6986,7 +7025,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6994,6 +7032,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7388,7 +7427,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7396,6 +7434,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7680,7 +7719,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7688,6 +7726,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8034,7 +8073,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8042,6 +8080,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8389,7 +8428,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8397,6 +8435,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8679,7 +8718,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8687,6 +8725,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9023,7 +9062,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9031,6 +9069,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9375,7 +9414,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9383,6 +9421,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9666,7 +9705,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9674,6 +9712,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10018,7 +10057,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10026,6 +10064,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10362,7 +10401,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10370,6 +10408,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10653,7 +10692,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10661,6 +10699,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11004,7 +11043,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11012,6 +11050,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11351,7 +11390,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11359,6 +11397,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11698,7 +11737,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11706,6 +11744,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11979,7 +12018,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11987,6 +12025,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12327,7 +12366,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12335,6 +12373,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12675,7 +12714,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12683,6 +12721,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12956,7 +12995,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12964,6 +13002,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13245,7 +13284,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13253,6 +13291,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13534,7 +13573,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13542,6 +13580,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -13815,7 +13854,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -13823,6 +13861,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14104,7 +14143,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14112,6 +14150,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14484,7 +14523,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14492,6 +14530,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14773,7 +14812,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14781,6 +14819,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15054,7 +15093,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15062,6 +15100,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15433,7 +15472,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15441,6 +15479,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15783,7 +15822,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15791,6 +15829,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16336,7 +16375,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -16344,6 +16382,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16894,7 +16933,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -16902,6 +16940,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -17246,7 +17285,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -17254,6 +17292,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -49863,7 +49902,7 @@
       <c r="D3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="36" t="s">
         <v>50</v>
       </c>
       <c r="F3" s="4" t="s">
@@ -49878,7 +49917,7 @@
       <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="37" t="s">
         <v>42</v>
       </c>
       <c r="F4" s="4" t="s">
@@ -49908,7 +49947,7 @@
       <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="36" t="s">
         <v>51</v>
       </c>
       <c r="F6" s="4" t="s">
@@ -49923,7 +49962,7 @@
       <c r="D7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="36" t="s">
         <v>52</v>
       </c>
       <c r="F7" s="4" t="s">
@@ -49953,7 +49992,7 @@
       <c r="D9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="40" t="s">
         <v>43</v>
       </c>
       <c r="F9" s="4"/>
@@ -49968,7 +50007,7 @@
       <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="40" t="s">
         <v>53</v>
       </c>
       <c r="F10" s="4"/>
@@ -49980,7 +50019,9 @@
       <c r="D11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="8"/>
+      <c r="E11" s="36" t="s">
+        <v>55</v>
+      </c>
       <c r="F11" s="4" t="s">
         <v>27</v>
       </c>
@@ -50034,7 +50075,7 @@
       <c r="D15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="38" t="s">
         <v>54</v>
       </c>
       <c r="F15" s="4" t="s">
@@ -50066,7 +50107,7 @@
       <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="38" t="s">
         <v>46</v>
       </c>
       <c r="F17" s="4" t="s">
@@ -50083,7 +50124,7 @@
       <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="38" t="s">
         <v>48</v>
       </c>
       <c r="F18" s="4" t="s">
@@ -50100,7 +50141,7 @@
       <c r="D19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="39" t="s">
         <v>43</v>
       </c>
       <c r="F19" s="4"/>
@@ -50112,7 +50153,7 @@
       <c r="D20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="38" t="s">
         <v>55</v>
       </c>
       <c r="F20" s="4" t="s">
@@ -53436,425 +53477,436 @@
     </row>
     <row r="24" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18"/>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32" t="s">
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32" t="s">
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="R24" s="32" t="s">
+      <c r="J24" s="35"/>
+      <c r="K24" s="35"/>
+      <c r="L24" s="35"/>
+      <c r="M24" s="35"/>
+      <c r="R24" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="S24" s="32"/>
-      <c r="T24" s="32"/>
-      <c r="U24" s="32"/>
-      <c r="V24" s="32"/>
-      <c r="W24" s="32" t="s">
+      <c r="S24" s="35"/>
+      <c r="T24" s="35"/>
+      <c r="U24" s="35"/>
+      <c r="V24" s="35"/>
+      <c r="W24" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="X24" s="32"/>
-      <c r="Y24" s="32" t="s">
+      <c r="X24" s="35"/>
+      <c r="Y24" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="Z24" s="32"/>
-      <c r="AA24" s="32"/>
-      <c r="AB24" s="32"/>
-      <c r="AC24" s="32"/>
+      <c r="Z24" s="35"/>
+      <c r="AA24" s="35"/>
+      <c r="AB24" s="35"/>
+      <c r="AC24" s="35"/>
     </row>
     <row r="25" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-      <c r="T25" s="32"/>
-      <c r="U25" s="32"/>
-      <c r="V25" s="32"/>
-      <c r="W25" s="32"/>
-      <c r="X25" s="32"/>
-      <c r="Y25" s="32"/>
-      <c r="Z25" s="32"/>
-      <c r="AA25" s="32"/>
-      <c r="AB25" s="32"/>
-      <c r="AC25" s="32"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="35"/>
+      <c r="K25" s="35"/>
+      <c r="L25" s="35"/>
+      <c r="M25" s="35"/>
+      <c r="R25" s="35"/>
+      <c r="S25" s="35"/>
+      <c r="T25" s="35"/>
+      <c r="U25" s="35"/>
+      <c r="V25" s="35"/>
+      <c r="W25" s="35"/>
+      <c r="X25" s="35"/>
+      <c r="Y25" s="35"/>
+      <c r="Z25" s="35"/>
+      <c r="AA25" s="35"/>
+      <c r="AB25" s="35"/>
+      <c r="AC25" s="35"/>
     </row>
     <row r="26" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="R26" s="33" t="s">
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34"/>
+      <c r="R26" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="S26" s="33"/>
-      <c r="T26" s="33"/>
-      <c r="U26" s="33"/>
-      <c r="V26" s="33"/>
-      <c r="W26" s="33"/>
-      <c r="X26" s="33"/>
-      <c r="Y26" s="33"/>
-      <c r="Z26" s="33"/>
-      <c r="AA26" s="33"/>
-      <c r="AB26" s="33"/>
-      <c r="AC26" s="33"/>
+      <c r="S26" s="34"/>
+      <c r="T26" s="34"/>
+      <c r="U26" s="34"/>
+      <c r="V26" s="34"/>
+      <c r="W26" s="34"/>
+      <c r="X26" s="34"/>
+      <c r="Y26" s="34"/>
+      <c r="Z26" s="34"/>
+      <c r="AA26" s="34"/>
+      <c r="AB26" s="34"/>
+      <c r="AC26" s="34"/>
     </row>
     <row r="27" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="33" t="s">
         <v>72</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
       <c r="D27" s="20"/>
-      <c r="Q27" s="31" t="s">
+      <c r="Q27" s="33" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A28" s="31"/>
-      <c r="Q28" s="31"/>
+      <c r="A28" s="33"/>
+      <c r="Q28" s="33"/>
     </row>
     <row r="29" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A29" s="31"/>
-      <c r="Q29" s="31"/>
+      <c r="A29" s="33"/>
+      <c r="Q29" s="33"/>
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A30" s="31"/>
-      <c r="Q30" s="31"/>
+      <c r="A30" s="33"/>
+      <c r="Q30" s="33"/>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A31" s="31"/>
-      <c r="Q31" s="31"/>
+      <c r="A31" s="33"/>
+      <c r="Q31" s="33"/>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A32" s="31"/>
-      <c r="Q32" s="31"/>
+      <c r="A32" s="33"/>
+      <c r="Q32" s="33"/>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="23"/>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="33"/>
-      <c r="J33" s="33"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="34"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
       <c r="Q33" s="23"/>
-      <c r="R33" s="33" t="s">
+      <c r="R33" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="S33" s="33"/>
-      <c r="T33" s="33"/>
-      <c r="U33" s="33"/>
-      <c r="V33" s="33"/>
-      <c r="W33" s="33"/>
-      <c r="X33" s="33"/>
-      <c r="Y33" s="33"/>
-      <c r="Z33" s="33"/>
-      <c r="AA33" s="33"/>
-      <c r="AB33" s="33"/>
-      <c r="AC33" s="33"/>
+      <c r="S33" s="34"/>
+      <c r="T33" s="34"/>
+      <c r="U33" s="34"/>
+      <c r="V33" s="34"/>
+      <c r="W33" s="34"/>
+      <c r="X33" s="34"/>
+      <c r="Y33" s="34"/>
+      <c r="Z33" s="34"/>
+      <c r="AA33" s="34"/>
+      <c r="AB33" s="34"/>
+      <c r="AC33" s="34"/>
     </row>
     <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
+      <c r="A34" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="Q34" s="31" t="s">
+      <c r="Q34" s="33" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A35" s="31"/>
-      <c r="Q35" s="31"/>
+      <c r="A35" s="33"/>
+      <c r="Q35" s="33"/>
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="Q36" s="31"/>
+      <c r="A36" s="33"/>
+      <c r="Q36" s="33"/>
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A37" s="31"/>
-      <c r="Q37" s="31"/>
+      <c r="A37" s="33"/>
+      <c r="Q37" s="33"/>
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A38" s="31"/>
-      <c r="Q38" s="31"/>
+      <c r="A38" s="33"/>
+      <c r="Q38" s="33"/>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-      <c r="Q39" s="31"/>
+      <c r="A39" s="33"/>
+      <c r="Q39" s="33"/>
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A40" s="31"/>
-      <c r="R40" s="33" t="s">
+      <c r="A40" s="33"/>
+      <c r="R40" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="S40" s="33"/>
-      <c r="T40" s="33"/>
-      <c r="U40" s="33"/>
-      <c r="V40" s="33"/>
-      <c r="W40" s="33"/>
-      <c r="X40" s="33"/>
-      <c r="Y40" s="33"/>
-      <c r="Z40" s="33"/>
-      <c r="AA40" s="33"/>
-      <c r="AB40" s="33"/>
-      <c r="AC40" s="33"/>
+      <c r="S40" s="34"/>
+      <c r="T40" s="34"/>
+      <c r="U40" s="34"/>
+      <c r="V40" s="34"/>
+      <c r="W40" s="34"/>
+      <c r="X40" s="34"/>
+      <c r="Y40" s="34"/>
+      <c r="Z40" s="34"/>
+      <c r="AA40" s="34"/>
+      <c r="AB40" s="34"/>
+      <c r="AC40" s="34"/>
     </row>
     <row r="41" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A41" s="31"/>
-      <c r="Q41" s="31" t="s">
+      <c r="A41" s="33"/>
+      <c r="Q41" s="33" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="23"/>
-      <c r="B42" s="33" t="s">
+      <c r="B42" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
-      <c r="M42" s="33"/>
-      <c r="Q42" s="31"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="34"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="34"/>
+      <c r="J42" s="34"/>
+      <c r="K42" s="34"/>
+      <c r="L42" s="34"/>
+      <c r="M42" s="34"/>
+      <c r="Q42" s="33"/>
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A43" s="31" t="s">
+      <c r="A43" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="Q43" s="31"/>
+      <c r="Q43" s="33"/>
     </row>
     <row r="44" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A44" s="31"/>
-      <c r="Q44" s="31"/>
+      <c r="A44" s="33"/>
+      <c r="Q44" s="33"/>
     </row>
     <row r="45" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A45" s="31"/>
+      <c r="A45" s="33"/>
       <c r="P45" s="27"/>
-      <c r="Q45" s="31"/>
+      <c r="Q45" s="33"/>
     </row>
     <row r="46" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A46" s="31"/>
-      <c r="Q46" s="31"/>
+      <c r="A46" s="33"/>
+      <c r="Q46" s="33"/>
     </row>
     <row r="47" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A47" s="31"/>
-      <c r="Q47" s="31" t="s">
+      <c r="A47" s="33"/>
+      <c r="Q47" s="33" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A48" s="31"/>
-      <c r="Q48" s="31"/>
+      <c r="A48" s="33"/>
+      <c r="Q48" s="33"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
-      <c r="B49" s="33" t="s">
+      <c r="B49" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C49" s="33"/>
-      <c r="D49" s="33"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
-      <c r="J49" s="33"/>
-      <c r="K49" s="33"/>
-      <c r="L49" s="33"/>
-      <c r="M49" s="33"/>
-      <c r="Q49" s="31"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="34"/>
+      <c r="E49" s="34"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="34"/>
+      <c r="H49" s="34"/>
+      <c r="I49" s="34"/>
+      <c r="J49" s="34"/>
+      <c r="K49" s="34"/>
+      <c r="L49" s="34"/>
+      <c r="M49" s="34"/>
+      <c r="Q49" s="33"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="31" t="s">
+      <c r="A50" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="Q50" s="31"/>
+      <c r="Q50" s="33"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="31"/>
-      <c r="Q51" s="31"/>
+      <c r="A51" s="33"/>
+      <c r="Q51" s="33"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="31"/>
-      <c r="Q52" s="31"/>
+      <c r="A52" s="33"/>
+      <c r="Q52" s="33"/>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="31"/>
+      <c r="A53" s="33"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="31"/>
+      <c r="A54" s="33"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A55" s="31"/>
+      <c r="A55" s="33"/>
     </row>
     <row r="57" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="35" t="s">
+      <c r="B57" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="35"/>
-      <c r="H57" s="35"/>
-      <c r="I57" s="35"/>
-      <c r="J57" s="35"/>
-      <c r="K57" s="35"/>
-      <c r="L57" s="35"/>
-      <c r="M57" s="35"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="31"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="31"/>
+      <c r="G57" s="31"/>
+      <c r="H57" s="31"/>
+      <c r="I57" s="31"/>
+      <c r="J57" s="31"/>
+      <c r="K57" s="31"/>
+      <c r="L57" s="31"/>
+      <c r="M57" s="31"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B58" s="35"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
-      <c r="G58" s="35"/>
-      <c r="H58" s="35"/>
-      <c r="I58" s="35"/>
-      <c r="J58" s="35"/>
-      <c r="K58" s="35"/>
-      <c r="L58" s="35"/>
-      <c r="M58" s="35"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="31"/>
+      <c r="E58" s="31"/>
+      <c r="F58" s="31"/>
+      <c r="G58" s="31"/>
+      <c r="H58" s="31"/>
+      <c r="I58" s="31"/>
+      <c r="J58" s="31"/>
+      <c r="K58" s="31"/>
+      <c r="L58" s="31"/>
+      <c r="M58" s="31"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B59" s="34" t="s">
+      <c r="B59" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="34"/>
-      <c r="D59" s="34"/>
-      <c r="E59" s="34"/>
-      <c r="F59" s="34"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="34"/>
-      <c r="I59" s="34"/>
-      <c r="J59" s="34"/>
-      <c r="K59" s="34"/>
-      <c r="L59" s="34"/>
-      <c r="M59" s="34"/>
+      <c r="C59" s="32"/>
+      <c r="D59" s="32"/>
+      <c r="E59" s="32"/>
+      <c r="F59" s="32"/>
+      <c r="G59" s="32"/>
+      <c r="H59" s="32"/>
+      <c r="I59" s="32"/>
+      <c r="J59" s="32"/>
+      <c r="K59" s="32"/>
+      <c r="L59" s="32"/>
+      <c r="M59" s="32"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B60" s="34"/>
-      <c r="C60" s="34"/>
-      <c r="D60" s="34"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
-      <c r="J60" s="34"/>
-      <c r="K60" s="34"/>
-      <c r="L60" s="34"/>
-      <c r="M60" s="34"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="32"/>
+      <c r="D60" s="32"/>
+      <c r="E60" s="32"/>
+      <c r="F60" s="32"/>
+      <c r="G60" s="32"/>
+      <c r="H60" s="32"/>
+      <c r="I60" s="32"/>
+      <c r="J60" s="32"/>
+      <c r="K60" s="32"/>
+      <c r="L60" s="32"/>
+      <c r="M60" s="32"/>
     </row>
     <row r="66" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R66" s="35" t="s">
+      <c r="R66" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="S66" s="35"/>
-      <c r="T66" s="35"/>
-      <c r="U66" s="35"/>
-      <c r="V66" s="35"/>
-      <c r="W66" s="35"/>
-      <c r="X66" s="35"/>
-      <c r="Y66" s="35"/>
-      <c r="Z66" s="35"/>
-      <c r="AA66" s="35"/>
-      <c r="AB66" s="35"/>
-      <c r="AC66" s="35"/>
+      <c r="S66" s="31"/>
+      <c r="T66" s="31"/>
+      <c r="U66" s="31"/>
+      <c r="V66" s="31"/>
+      <c r="W66" s="31"/>
+      <c r="X66" s="31"/>
+      <c r="Y66" s="31"/>
+      <c r="Z66" s="31"/>
+      <c r="AA66" s="31"/>
+      <c r="AB66" s="31"/>
+      <c r="AC66" s="31"/>
     </row>
     <row r="67" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R67" s="35"/>
-      <c r="S67" s="35"/>
-      <c r="T67" s="35"/>
-      <c r="U67" s="35"/>
-      <c r="V67" s="35"/>
-      <c r="W67" s="35"/>
-      <c r="X67" s="35"/>
-      <c r="Y67" s="35"/>
-      <c r="Z67" s="35"/>
-      <c r="AA67" s="35"/>
-      <c r="AB67" s="35"/>
-      <c r="AC67" s="35"/>
+      <c r="R67" s="31"/>
+      <c r="S67" s="31"/>
+      <c r="T67" s="31"/>
+      <c r="U67" s="31"/>
+      <c r="V67" s="31"/>
+      <c r="W67" s="31"/>
+      <c r="X67" s="31"/>
+      <c r="Y67" s="31"/>
+      <c r="Z67" s="31"/>
+      <c r="AA67" s="31"/>
+      <c r="AB67" s="31"/>
+      <c r="AC67" s="31"/>
     </row>
     <row r="68" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R68" s="34" t="s">
+      <c r="R68" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="S68" s="34"/>
-      <c r="T68" s="34"/>
-      <c r="U68" s="34"/>
-      <c r="V68" s="34"/>
-      <c r="W68" s="34"/>
-      <c r="X68" s="34"/>
-      <c r="Y68" s="34"/>
-      <c r="Z68" s="34"/>
-      <c r="AA68" s="34"/>
-      <c r="AB68" s="34"/>
-      <c r="AC68" s="34"/>
+      <c r="S68" s="32"/>
+      <c r="T68" s="32"/>
+      <c r="U68" s="32"/>
+      <c r="V68" s="32"/>
+      <c r="W68" s="32"/>
+      <c r="X68" s="32"/>
+      <c r="Y68" s="32"/>
+      <c r="Z68" s="32"/>
+      <c r="AA68" s="32"/>
+      <c r="AB68" s="32"/>
+      <c r="AC68" s="32"/>
     </row>
     <row r="69" spans="18:29" x14ac:dyDescent="0.25">
-      <c r="R69" s="34"/>
-      <c r="S69" s="34"/>
-      <c r="T69" s="34"/>
-      <c r="U69" s="34"/>
-      <c r="V69" s="34"/>
-      <c r="W69" s="34"/>
-      <c r="X69" s="34"/>
-      <c r="Y69" s="34"/>
-      <c r="Z69" s="34"/>
-      <c r="AA69" s="34"/>
-      <c r="AB69" s="34"/>
-      <c r="AC69" s="34"/>
+      <c r="R69" s="32"/>
+      <c r="S69" s="32"/>
+      <c r="T69" s="32"/>
+      <c r="U69" s="32"/>
+      <c r="V69" s="32"/>
+      <c r="W69" s="32"/>
+      <c r="X69" s="32"/>
+      <c r="Y69" s="32"/>
+      <c r="Z69" s="32"/>
+      <c r="AA69" s="32"/>
+      <c r="AB69" s="32"/>
+      <c r="AC69" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="Q34:Q39"/>
+    <mergeCell ref="Q41:Q46"/>
+    <mergeCell ref="Q47:Q52"/>
+    <mergeCell ref="B49:M49"/>
+    <mergeCell ref="B59:M60"/>
+    <mergeCell ref="B57:M58"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="I24:M25"/>
+    <mergeCell ref="Q27:Q32"/>
+    <mergeCell ref="B26:M26"/>
+    <mergeCell ref="B33:M33"/>
     <mergeCell ref="R66:AC67"/>
     <mergeCell ref="R68:AC69"/>
     <mergeCell ref="R21:AC23"/>
@@ -53871,17 +53923,6 @@
     <mergeCell ref="W24:X25"/>
     <mergeCell ref="E24:H25"/>
     <mergeCell ref="A50:A55"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="I24:M25"/>
-    <mergeCell ref="Q27:Q32"/>
-    <mergeCell ref="B26:M26"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="Q34:Q39"/>
-    <mergeCell ref="Q41:Q46"/>
-    <mergeCell ref="Q47:Q52"/>
-    <mergeCell ref="B49:M49"/>
-    <mergeCell ref="B59:M60"/>
-    <mergeCell ref="B57:M58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>